<commit_message>
Added Updates to Customer_Feedback Ex2A and Added Ex4b
</commit_message>
<xml_diff>
--- a/week-01/Red Robins Customer Feedback Review(1-5).xlsx
+++ b/week-01/Red Robins Customer Feedback Review(1-5).xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30610"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -16,9 +16,9 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="22" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -42,6 +42,24 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="44">
   <si>
+    <t>Row Labels</t>
+  </si>
+  <si>
+    <t>Count of Name</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
+  <si>
+    <t>Sum of ID</t>
+  </si>
+  <si>
+    <t>Chicken Wings</t>
+  </si>
+  <si>
+    <t>Delectable Desserts</t>
+  </si>
+  <si>
     <t>ID</t>
   </si>
   <si>
@@ -51,6 +69,9 @@
     <t>Completion time</t>
   </si>
   <si>
+    <t>Time to complete</t>
+  </si>
+  <si>
     <t>Email</t>
   </si>
   <si>
@@ -99,9 +120,6 @@
     <t>Better than expected</t>
   </si>
   <si>
-    <t>Chicken Wings</t>
-  </si>
-  <si>
     <t>Dirty Soda</t>
   </si>
   <si>
@@ -144,9 +162,6 @@
     <t>denae mendez</t>
   </si>
   <si>
-    <t>Delectable Desserts</t>
-  </si>
-  <si>
     <t>This looks great! I almost thought this was an actual survey from red robin's! I do have one suggestion though if you are open to receiving feedback. Maybe this question should be optional (^_^;)</t>
   </si>
   <si>
@@ -157,21 +172,6 @@
   </si>
   <si>
     <t>Make those wings hotter! I could eat those for breakfast, lunch and dinner!</t>
-  </si>
-  <si>
-    <t>Time to complete</t>
-  </si>
-  <si>
-    <t>Row Labels</t>
-  </si>
-  <si>
-    <t>Grand Total</t>
-  </si>
-  <si>
-    <t>Count of Name</t>
-  </si>
-  <si>
-    <t>Sum of ID</t>
   </si>
 </sst>
 </file>
@@ -180,9 +180,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="m/d/yy\ h:mm:ss"/>
-    <numFmt numFmtId="166" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -211,11 +211,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="45" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -257,39 +256,6 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="m/d/yy\ h:mm:ss"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="28" formatCode="mm:ss"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="28" formatCode="mm:ss"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
@@ -321,6 +287,39 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="m/d/yy\ h:mm:ss"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="m/d/yy\ h:mm:ss"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="28" formatCode="mm:ss"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="28" formatCode="mm:ss"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -449,8 +448,7 @@
           </a:effectLst>
         </c:spPr>
         <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="6"/>
+          <c:symbol val="none"/>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
@@ -491,6 +489,78 @@
           </c:extLst>
         </c:dLbl>
       </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst>
+            <a:outerShdw blurRad="317500" algn="ctr" rotWithShape="0">
+              <a:prstClr val="black">
+                <a:alpha val="25000"/>
+              </a:prstClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="3"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst>
+            <a:outerShdw blurRad="317500" algn="ctr" rotWithShape="0">
+              <a:prstClr val="black">
+                <a:alpha val="25000"/>
+              </a:prstClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="4"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst>
+            <a:outerShdw blurRad="317500" algn="ctr" rotWithShape="0">
+              <a:prstClr val="black">
+                <a:alpha val="25000"/>
+              </a:prstClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="5"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst>
+            <a:outerShdw blurRad="317500" algn="ctr" rotWithShape="0">
+              <a:prstClr val="black">
+                <a:alpha val="25000"/>
+              </a:prstClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </c:spPr>
+      </c:pivotFmt>
     </c:pivotFmts>
     <c:plotArea>
       <c:layout/>
@@ -528,6 +598,11 @@
                 </a:outerShdw>
               </a:effectLst>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-2093-4AE8-9389-69654A122BD0}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -547,6 +622,11 @@
                 </a:outerShdw>
               </a:effectLst>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-2093-4AE8-9389-69654A122BD0}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -566,6 +646,11 @@
                 </a:outerShdw>
               </a:effectLst>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-2093-4AE8-9389-69654A122BD0}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="3"/>
@@ -585,6 +670,11 @@
                 </a:outerShdw>
               </a:effectLst>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-2093-4AE8-9389-69654A122BD0}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dLbls>
             <c:spPr>
@@ -2428,10 +2518,10 @@
     <cacheField name="ID" numFmtId="0">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="5"/>
     </cacheField>
-    <cacheField name="Start time" numFmtId="166">
+    <cacheField name="Start time" numFmtId="165">
       <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-10-14T23:14:04" maxDate="2026-10-16T18:37:34"/>
     </cacheField>
-    <cacheField name="Completion time" numFmtId="166">
+    <cacheField name="Completion time" numFmtId="165">
       <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-10-14T23:16:14" maxDate="2026-10-16T18:38:48"/>
     </cacheField>
     <cacheField name="Time to complete" numFmtId="45">
@@ -2495,6 +2585,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
       <x14:pivotCacheDefinition/>
+    </ext>
+    <ext xmlns:xlpdsc="http://schemas.microsoft.com/office/spreadsheetml/2026/pivotDataSourceClean" uri="{F4336242-56EE-4DD3-A5F7-E900642BF6E9}">
+      <xlpdsc:dataSourceClean>1</xlpdsc:dataSourceClean>
     </ext>
   </extLst>
 </pivotCacheDefinition>
@@ -2601,12 +2694,12 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E77F246D-45C2-4298-B4E5-DC2EAF4EE05D}" name="PivotTable6" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E77F246D-45C2-4298-B4E5-DC2EAF4EE05D}" name="PivotTable6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A17:B20" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="17">
     <pivotField dataField="1" showAll="0"/>
-    <pivotField numFmtId="166" showAll="0"/>
-    <pivotField numFmtId="166" showAll="0"/>
+    <pivotField numFmtId="165" showAll="0"/>
+    <pivotField numFmtId="165" showAll="0"/>
     <pivotField numFmtId="45" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -2685,12 +2778,12 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{59447474-96E4-4D34-B35E-A45EE0F33C4D}" name="PivotTable5" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{59447474-96E4-4D34-B35E-A45EE0F33C4D}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
   <location ref="A1:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="17">
     <pivotField showAll="0"/>
-    <pivotField numFmtId="166" showAll="0"/>
-    <pivotField numFmtId="166" showAll="0"/>
+    <pivotField numFmtId="165" showAll="0"/>
+    <pivotField numFmtId="165" showAll="0"/>
     <pivotField numFmtId="45" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
@@ -2740,12 +2833,60 @@
   <dataFields count="1">
     <dataField name="Count of Name" fld="5" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
-  <chartFormats count="1">
+  <chartFormats count="5">
     <chartFormat chart="0" format="1" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="2">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="10" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="3">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="10" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="4">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="10" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="5">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="10" count="1" selected="0">
+            <x v="3"/>
           </reference>
         </references>
       </pivotArea>
@@ -2767,44 +2908,44 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:Q7" totalsRowCount="1">
   <autoFilter ref="A1:Q6" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" dataDxfId="20" totalsRowDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Start time" dataDxfId="19" totalsRowDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Completion time" dataDxfId="18" totalsRowDxfId="14"/>
-    <tableColumn id="17" xr3:uid="{BAE919A1-D624-44B3-BA77-32A8BA353F8E}" name="Time to complete" totalsRowFunction="custom" dataDxfId="17" totalsRowDxfId="13">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" dataDxfId="32" totalsRowDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Start time" dataDxfId="30" totalsRowDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Completion time" dataDxfId="28" totalsRowDxfId="29"/>
+    <tableColumn id="17" xr3:uid="{BAE919A1-D624-44B3-BA77-32A8BA353F8E}" name="Time to complete" totalsRowFunction="custom" dataDxfId="26" totalsRowDxfId="27">
       <calculatedColumnFormula>C2-B2</calculatedColumnFormula>
       <totalsRowFormula>AVERAGE(D2:D6)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Email" dataDxfId="33" totalsRowDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Name" dataDxfId="32" totalsRowDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Last modified time" dataDxfId="31" totalsRowDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="How would you rate the overall quality of your meal today?" totalsRowFunction="custom" dataDxfId="30" totalsRowDxfId="9">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Email" dataDxfId="24" totalsRowDxfId="25"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Name" dataDxfId="22" totalsRowDxfId="23"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Last modified time" dataDxfId="20" totalsRowDxfId="21"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="How would you rate the overall quality of your meal today?" totalsRowFunction="custom" dataDxfId="18" totalsRowDxfId="19">
       <totalsRowFormula>SUM(COUNTIF(Table1[How would you rate the overall quality of your meal today?],"As expected"),COUNTIF(Table1[How would you rate the overall quality of your meal today?],"Better than expected"))</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Please indicate your overall satisfaction with Red Robins item selections." totalsRowFunction="custom" dataDxfId="29" totalsRowDxfId="8">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Please indicate your overall satisfaction with Red Robins item selections." totalsRowFunction="custom" dataDxfId="16" totalsRowDxfId="17">
       <totalsRowFormula>AVERAGE(I2:I6)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Quick! Which is your go to Red Robin guilty pleasure?" totalsRowFunction="custom" dataDxfId="28" totalsRowDxfId="7">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Quick! Which is your go to Red Robin guilty pleasure?" totalsRowFunction="custom" dataDxfId="14" totalsRowDxfId="15">
       <totalsRowFormula>SUM(COUNTIF(Table1[Quick! Which is your go to Red Robin guilty pleasure?],"Chicken Wings"),COUNTIF(Table1[Quick! Which is your go to Red Robin guilty pleasure?],"Delectable Desserts"))</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="How likely are you to recommend us to the friends and family?" totalsRowFunction="custom" dataDxfId="27" totalsRowDxfId="6">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="How likely are you to recommend us to the friends and family?" totalsRowFunction="custom" dataDxfId="12" totalsRowDxfId="13">
       <totalsRowFormula>AVERAGE(K2:K6)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="There can only be one." totalsRowFunction="custom" dataDxfId="26" totalsRowDxfId="5">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="There can only be one." totalsRowFunction="custom" dataDxfId="10" totalsRowDxfId="11">
       <totalsRowFormula>SUM(COUNTIF(Table1[There can only be one.],"Dirt Soda"),COUNTIF(Table1[There can only be one.],"Gourmet Milkshake"))</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Are you a Red Robin Rewards Member?" totalsRowFunction="custom" dataDxfId="25" totalsRowDxfId="4">
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Are you a Red Robin Rewards Member?" totalsRowFunction="custom" dataDxfId="8" totalsRowDxfId="9">
       <totalsRowFormula>SUM(COUNTIF(Table1[Are you a Red Robin Rewards Member?],"I'd like to sign up and receive my free appetizer alongside dipping fries in campfire sauce!"))</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="How likely are you to return back to this Red Robin location?" totalsRowFunction="custom" dataDxfId="24" totalsRowDxfId="3">
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="How likely are you to return back to this Red Robin location?" totalsRowFunction="custom" dataDxfId="6" totalsRowDxfId="7">
       <totalsRowFormula>AVERAGE(N2:N6)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="How satisfied are you with the manner of time in which you received your order?" totalsRowFunction="custom" dataDxfId="23" totalsRowDxfId="2">
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="How satisfied are you with the manner of time in which you received your order?" totalsRowFunction="custom" dataDxfId="4" totalsRowDxfId="5">
       <totalsRowFormula>AVERAGE(O2:O6)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="How well would you rate your service and experience with Red Robins Today?" totalsRowFunction="custom" dataDxfId="22" totalsRowDxfId="1">
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="How well would you rate your service and experience with Red Robins Today?" totalsRowFunction="custom" dataDxfId="2" totalsRowDxfId="3">
       <totalsRowFormula>AVERAGE(P2:P6)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Do you have any feedback, comments, or suggestions you would like to provide?" dataDxfId="21" totalsRowDxfId="0"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Do you have any feedback, comments, or suggestions you would like to provide?" dataDxfId="0" totalsRowDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3108,91 +3249,91 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB5CFF7E-92DD-49D2-8BD6-E52DD113501B}">
   <dimension ref="A1:B20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
-        <v>40</v>
+    <row r="1" spans="1:2">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>42</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="6">
+    <row r="2" spans="1:2">
+      <c r="A2" s="5">
         <v>7</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="6">
+    <row r="3" spans="1:2">
+      <c r="A3" s="5">
         <v>8</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="6">
+    <row r="4" spans="1:2">
+      <c r="A4" s="5">
         <v>9</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="6">
+    <row r="5" spans="1:2">
+      <c r="A5" s="5">
         <v>10</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6" s="2">
+    <row r="6" spans="1:2">
+      <c r="A6" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6">
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="5" t="s">
-        <v>40</v>
+    <row r="17" spans="1:2">
+      <c r="A17" s="4" t="s">
+        <v>0</v>
       </c>
       <c r="B17" t="s">
-        <v>43</v>
+        <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="2">
+    <row r="18" spans="1:2">
+      <c r="A18" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18">
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="B19" s="2">
+    <row r="19" spans="1:2">
+      <c r="A19" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19">
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B20" s="2">
+    <row r="20" spans="1:2">
+      <c r="A20" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B20">
         <v>15</v>
       </c>
     </row>
@@ -3205,106 +3346,106 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20" style="4" customWidth="1"/>
+    <col min="4" max="4" width="20" style="3" customWidth="1"/>
     <col min="5" max="17" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17">
       <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
+        <v>6</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>39</v>
+        <v>8</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="E1" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="G1" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="H1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="I1" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="K1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="L1" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="M1" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="N1" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="O1" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="P1" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="Q1" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <v>46309.968101851853</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="2">
         <v>46309.969606481478</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <f t="shared" ref="D2:D6" si="0">C2-B2</f>
         <v>1.5046296248328872E-3</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="F2" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="G2" s="1"/>
       <c r="H2" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="I2">
         <v>4</v>
       </c>
       <c r="J2" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K2">
         <v>9</v>
       </c>
       <c r="L2" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="M2" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="N2">
         <v>10</v>
@@ -3316,47 +3457,47 @@
         <v>5</v>
       </c>
       <c r="Q2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>46310.355162037034</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>46310.380810185183</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="3">
         <f t="shared" si="0"/>
         <v>2.5648148148320615E-2</v>
       </c>
       <c r="E3" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G3" s="1"/>
       <c r="H3" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="I3">
         <v>5</v>
       </c>
       <c r="J3" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K3">
         <v>10</v>
       </c>
       <c r="L3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="M3" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="N3">
         <v>10</v>
@@ -3368,47 +3509,47 @@
         <v>5</v>
       </c>
       <c r="Q3" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>46311.563969907409</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>46311.564699074072</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="3">
         <f t="shared" si="0"/>
         <v>7.2916666249511763E-4</v>
       </c>
       <c r="E4" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="F4" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="I4">
         <v>5</v>
       </c>
       <c r="J4" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K4">
         <v>10</v>
       </c>
       <c r="L4" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="M4" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="N4">
         <v>10</v>
@@ -3420,47 +3561,47 @@
         <v>5</v>
       </c>
       <c r="Q4" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>46311.694710648146</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <v>46311.696759259263</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <f t="shared" si="0"/>
         <v>2.0486111170612276E-3</v>
       </c>
       <c r="E5" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="F5" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="G5" s="1"/>
       <c r="H5" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="I5">
         <v>3</v>
       </c>
       <c r="J5" t="s">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="K5">
         <v>7</v>
       </c>
       <c r="L5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="M5" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="N5">
         <v>6</v>
@@ -3472,47 +3613,47 @@
         <v>4</v>
       </c>
       <c r="Q5" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>46311.776087962964</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <v>46311.776944444442</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="3">
         <f t="shared" si="0"/>
         <v>8.5648147796746343E-4</v>
       </c>
       <c r="E6" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="F6" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="G6" s="1"/>
       <c r="H6" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="I6">
         <v>5</v>
       </c>
       <c r="J6" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="K6">
         <v>8</v>
       </c>
       <c r="L6" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="M6" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="N6">
         <v>10</v>
@@ -3524,56 +3665,52 @@
         <v>4</v>
       </c>
       <c r="Q6" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A7" s="2"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="4">
+    <row r="7" spans="1:17">
+      <c r="C7" s="2"/>
+      <c r="D7" s="3">
         <f>AVERAGE(D2:D6)</f>
         <v>6.1574074061354622E-3</v>
       </c>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
       <c r="G7" s="1"/>
-      <c r="H7" s="2">
+      <c r="H7">
         <f>SUM(COUNTIF(Table1[How would you rate the overall quality of your meal today?],"As expected"),COUNTIF(Table1[How would you rate the overall quality of your meal today?],"Better than expected"))</f>
         <v>5</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7">
         <f>AVERAGE(I2:I6)</f>
         <v>4.4000000000000004</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7">
         <f>SUM(COUNTIF(Table1[Quick! Which is your go to Red Robin guilty pleasure?],"Chicken Wings"),COUNTIF(Table1[Quick! Which is your go to Red Robin guilty pleasure?],"Delectable Desserts"))</f>
         <v>5</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7">
         <f>AVERAGE(K2:K6)</f>
         <v>8.8000000000000007</v>
       </c>
-      <c r="L7" s="2">
+      <c r="L7">
         <f>SUM(COUNTIF(Table1[There can only be one.],"Dirt Soda"),COUNTIF(Table1[There can only be one.],"Gourmet Milkshake"))</f>
         <v>3</v>
       </c>
-      <c r="M7" s="2">
+      <c r="M7">
         <f>SUM(COUNTIF(Table1[Are you a Red Robin Rewards Member?],"I'd like to sign up and receive my free appetizer alongside dipping fries in campfire sauce!"))</f>
         <v>3</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7">
         <f>AVERAGE(N2:N6)</f>
         <v>9.1999999999999993</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7">
         <f>AVERAGE(O2:O6)</f>
         <v>4.4000000000000004</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7">
         <f>AVERAGE(P2:P6)</f>
         <v>4.5999999999999996</v>
       </c>
-      <c r="Q7" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>